<commit_message>
Add and search edit finalized
</commit_message>
<xml_diff>
--- a/DB/Claim_Calling_Tracker1.1.xlsx
+++ b/DB/Claim_Calling_Tracker1.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Documents\GitHub\Caller_Tracker\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBA4F62D-EE6A-4C86-9FEE-4CABFA8F58FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6749EA4-5BA3-43C0-802D-93BE1400FD49}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="91">
   <si>
     <t>ClaimID</t>
   </si>
@@ -304,6 +304,9 @@
   </si>
   <si>
     <t>Query is not resolved.</t>
+  </si>
+  <si>
+    <t>No Answer recieved.</t>
   </si>
 </sst>
 </file>
@@ -415,8 +418,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblHistory" displayName="tblHistory" ref="A1:F10">
-  <autoFilter ref="A1:F10" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblHistory" displayName="tblHistory" ref="A1:F11">
+  <autoFilter ref="A1:F11" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="HistoryID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="ClaimID"/>
@@ -1254,7 +1257,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>671234</v>
       </c>
@@ -1286,7 +1289,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>4545</v>
       </c>
@@ -1318,7 +1321,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>121212</v>
       </c>
@@ -1338,7 +1341,7 @@
         <v>48</v>
       </c>
       <c r="G19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" t="s">
         <v>87</v>
@@ -1348,6 +1351,15 @@
       </c>
       <c r="J19" t="s">
         <v>49</v>
+      </c>
+      <c r="K19" s="4">
+        <v>46281.000972222224</v>
+      </c>
+      <c r="L19" t="s">
+        <v>49</v>
+      </c>
+      <c r="M19" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1361,7 +1373,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="16" customWidth="1"/>
@@ -1549,6 +1561,26 @@
         <v>69</v>
       </c>
       <c r="F10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>121212</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="4">
+        <v>46281.000972222224</v>
+      </c>
+      <c r="E11" t="s">
+        <v>90</v>
+      </c>
+      <c r="F11" t="s">
         <v>48</v>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker 0.4 is updated
</commit_message>
<xml_diff>
--- a/DB/Claim_Calling_Tracker1.1.xlsx
+++ b/DB/Claim_Calling_Tracker1.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Documents\GitHub\Caller_Tracker\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6749EA4-5BA3-43C0-802D-93BE1400FD49}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF7A97F-5515-4BBF-B4D5-99137DD03E18}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="93">
   <si>
     <t>ClaimID</t>
   </si>
@@ -307,6 +307,12 @@
   </si>
   <si>
     <t>No Answer recieved.</t>
+  </si>
+  <si>
+    <t>Abhilash</t>
+  </si>
+  <si>
+    <t>What is your name ?</t>
   </si>
 </sst>
 </file>
@@ -395,8 +401,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N19">
-  <autoFilter ref="A1:N19" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N20">
+  <autoFilter ref="A1:N20" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ClaimID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ClaimSite"/>
@@ -718,7 +724,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -1360,6 +1366,38 @@
       </c>
       <c r="M19" t="s">
         <v>90</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>454545</v>
+      </c>
+      <c r="B20" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" t="s">
+        <v>92</v>
+      </c>
+      <c r="E20" s="3">
+        <v>46282</v>
+      </c>
+      <c r="F20" t="s">
+        <v>48</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20" t="s">
+        <v>45</v>
+      </c>
+      <c r="I20" s="4">
+        <v>46281.322129629632</v>
+      </c>
+      <c r="J20" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
filter archieve is now working fine.
</commit_message>
<xml_diff>
--- a/DB/Claim_Calling_Tracker1.1.xlsx
+++ b/DB/Claim_Calling_Tracker1.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Documents\GitHub\Caller_Tracker\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE03D3C-52B0-4FD5-9A4F-3C2BDDBEE06B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC7ACE6D-9D1A-4C9F-B5A5-C149C680BAC8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="97">
   <si>
     <t>ClaimID</t>
   </si>
@@ -316,6 +316,15 @@
   </si>
   <si>
     <t>Testing Archieved</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>closed</t>
   </si>
 </sst>
 </file>
@@ -335,6 +344,7 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -404,8 +414,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N19">
-  <autoFilter ref="A1:N19" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tblClaims" displayName="tblClaims" ref="A1:N17">
+  <autoFilter ref="A1:N17" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ClaimID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ClaimSite"/>
@@ -427,8 +437,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblHistory" displayName="tblHistory" ref="A1:F8">
-  <autoFilter ref="A1:F8" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="tblHistory" displayName="tblHistory" ref="A1:F3">
+  <autoFilter ref="A1:F3" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="HistoryID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="ClaimID"/>
@@ -727,7 +737,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -787,21 +797,53 @@
         <v>13</v>
       </c>
     </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E2" s="3">
+        <v>46023</v>
+      </c>
+      <c r="F2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I2" s="4">
+        <v>46274.647858796299</v>
+      </c>
+      <c r="J2" t="s">
+        <v>49</v>
+      </c>
+    </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
         <v>45</v>
       </c>
       <c r="C3" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="E3" s="3">
-        <v>46023</v>
+        <v>46056</v>
       </c>
       <c r="F3" t="s">
         <v>48</v>
@@ -813,7 +855,7 @@
         <v>45</v>
       </c>
       <c r="I3" s="4">
-        <v>46274.647858796299</v>
+        <v>46274.685497685183</v>
       </c>
       <c r="J3" t="s">
         <v>49</v>
@@ -821,16 +863,16 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="C4" t="s">
         <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E4" s="3">
         <v>46056</v>
@@ -842,7 +884,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="I4" s="4">
         <v>46274.685497685183</v>
@@ -855,16 +897,16 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
         <v>56</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E5" s="3">
         <v>46056</v>
@@ -876,7 +918,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="I5" s="4">
         <v>46274.685497685183</v>
@@ -887,19 +929,19 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B6" t="s">
         <v>45</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E6" s="3">
-        <v>46056</v>
+        <v>46084</v>
       </c>
       <c r="F6" t="s">
         <v>48</v>
@@ -911,7 +953,7 @@
         <v>45</v>
       </c>
       <c r="I6" s="4">
-        <v>46274.685497685183</v>
+        <v>46274.687141203707</v>
       </c>
       <c r="J6" t="s">
         <v>49</v>
@@ -919,7 +961,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B7" t="s">
         <v>45</v>
@@ -951,7 +993,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B8" t="s">
         <v>45</v>
@@ -975,100 +1017,101 @@
         <v>45</v>
       </c>
       <c r="I8" s="4">
-        <v>46274.687141203707</v>
+        <v>46274.694351851853</v>
       </c>
       <c r="J8" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>65</v>
+      <c r="A9">
+        <v>11223344</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>85</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>84</v>
       </c>
       <c r="E9" s="3">
-        <v>46084</v>
+        <v>46275</v>
       </c>
       <c r="F9" t="s">
         <v>48</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>92</v>
       </c>
       <c r="I9" s="4">
-        <v>46274.694351851853</v>
+        <v>46275.459710648145</v>
       </c>
       <c r="J9" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="K9" s="4">
+        <v>46282.155381944445</v>
+      </c>
+      <c r="L9" t="s">
+        <v>49</v>
+      </c>
+      <c r="M9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="165" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>11223344</v>
+        <v>55555</v>
       </c>
       <c r="B10" t="s">
         <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>85</v>
-      </c>
-      <c r="D10" t="s">
-        <v>84</v>
+        <v>63</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>70</v>
       </c>
       <c r="E10" s="3">
-        <v>46275</v>
+        <v>46024</v>
       </c>
       <c r="F10" t="s">
         <v>48</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="I10" s="4">
-        <v>46275.459710648145</v>
+        <v>46275.575266203705</v>
       </c>
       <c r="J10" t="s">
         <v>49</v>
       </c>
-      <c r="K10" s="4">
-        <v>46282.155381944445</v>
-      </c>
-      <c r="L10" t="s">
-        <v>49</v>
-      </c>
-      <c r="M10" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="165" x14ac:dyDescent="0.25">
+      <c r="K10" s="4"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>55555</v>
+        <v>4141</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="E11" s="3">
-        <v>46024</v>
+        <v>414949</v>
       </c>
       <c r="F11" t="s">
         <v>48</v>
@@ -1077,10 +1120,10 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="I11" s="4">
-        <v>46275.575266203705</v>
+        <v>46276.548310185186</v>
       </c>
       <c r="J11" t="s">
         <v>49</v>
@@ -1088,21 +1131,21 @@
       <c r="K11" s="4"/>
       <c r="N11" s="4"/>
     </row>
-    <row r="12" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>1231234</v>
+        <v>6767</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="C12" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E12" s="3">
-        <v>46276</v>
+        <v>46023</v>
       </c>
       <c r="F12" t="s">
         <v>48</v>
@@ -1111,10 +1154,10 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>45</v>
+        <v>66</v>
       </c>
       <c r="I12" s="4">
-        <v>46276.529479166667</v>
+        <v>46276.552395833336</v>
       </c>
       <c r="J12" t="s">
         <v>49</v>
@@ -1124,19 +1167,19 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>4141</v>
+        <v>671234</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E13" s="3">
-        <v>414949</v>
+        <v>46023</v>
       </c>
       <c r="F13" t="s">
         <v>48</v>
@@ -1145,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H13" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="I13" s="4">
-        <v>46276.548310185186</v>
+        <v>46276.558287037034</v>
       </c>
       <c r="J13" t="s">
         <v>49</v>
@@ -1156,19 +1199,19 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>6767</v>
+        <v>4545</v>
       </c>
       <c r="B14" t="s">
         <v>66</v>
       </c>
       <c r="C14" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="D14" t="s">
         <v>76</v>
       </c>
       <c r="E14" s="3">
-        <v>46023</v>
+        <v>46055</v>
       </c>
       <c r="F14" t="s">
         <v>48</v>
@@ -1180,7 +1223,7 @@
         <v>66</v>
       </c>
       <c r="I14" s="4">
-        <v>46276.552395833336</v>
+        <v>46280.497164351851</v>
       </c>
       <c r="J14" t="s">
         <v>49</v>
@@ -1188,16 +1231,16 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>671234</v>
+        <v>121212</v>
       </c>
       <c r="B15" t="s">
-        <v>29</v>
+        <v>86</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="D15" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="E15" s="3">
         <v>46023</v>
@@ -1206,33 +1249,42 @@
         <v>48</v>
       </c>
       <c r="G15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" t="s">
-        <v>29</v>
+        <v>86</v>
       </c>
       <c r="I15" s="4">
-        <v>46276.558287037034</v>
+        <v>46280.982604166667</v>
       </c>
       <c r="J15" t="s">
         <v>49</v>
+      </c>
+      <c r="K15" s="4">
+        <v>46281.000972222224</v>
+      </c>
+      <c r="L15" t="s">
+        <v>49</v>
+      </c>
+      <c r="M15" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>4545</v>
+        <v>454545</v>
       </c>
       <c r="B16" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="C16" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="D16" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="E16" s="3">
-        <v>46055</v>
+        <v>46282</v>
       </c>
       <c r="F16" t="s">
         <v>48</v>
@@ -1241,93 +1293,48 @@
         <v>0</v>
       </c>
       <c r="H16" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="I16" s="4">
-        <v>46280.497164351851</v>
+        <v>46281.322129629632</v>
       </c>
       <c r="J16" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="K16" s="4"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>121212</v>
+        <v>1212</v>
       </c>
       <c r="B17" t="s">
         <v>86</v>
       </c>
       <c r="C17" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D17" t="s">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="E17" s="3">
-        <v>46023</v>
+        <v>46283</v>
       </c>
       <c r="F17" t="s">
         <v>48</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H17" t="s">
         <v>86</v>
       </c>
       <c r="I17" s="4">
-        <v>46280.982604166667</v>
+        <v>46282.215300925927</v>
       </c>
       <c r="J17" t="s">
         <v>49</v>
       </c>
-      <c r="K17" s="4">
-        <v>46281.000972222224</v>
-      </c>
-      <c r="L17" t="s">
-        <v>49</v>
-      </c>
-      <c r="M17" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18">
-        <v>454545</v>
-      </c>
-      <c r="B18" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" t="s">
-        <v>90</v>
-      </c>
-      <c r="D18" t="s">
-        <v>91</v>
-      </c>
-      <c r="E18" s="3">
-        <v>46282</v>
-      </c>
-      <c r="F18" t="s">
-        <v>48</v>
-      </c>
-      <c r="G18">
-        <v>0</v>
-      </c>
-      <c r="H18" t="s">
-        <v>45</v>
-      </c>
-      <c r="I18" s="4">
-        <v>46281.322129629632</v>
-      </c>
-      <c r="J18" t="s">
-        <v>49</v>
-      </c>
-      <c r="K18" s="4"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E19" s="3"/>
-      <c r="I19" s="4"/>
-      <c r="K19" s="4"/>
+      <c r="K17" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1340,7 +1347,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="16" customWidth="1"/>
@@ -1369,59 +1376,44 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D2" s="4"/>
+      <c r="A2">
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>11223344</v>
+      </c>
+      <c r="C2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="4">
+        <v>46277.185011574074</v>
+      </c>
+      <c r="E2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B3">
-        <v>11223344</v>
+        <v>121212</v>
       </c>
       <c r="C3" t="s">
         <v>49</v>
       </c>
       <c r="D3" s="4">
-        <v>46277.185011574074</v>
+        <v>46281.000972222224</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="F3" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>9</v>
-      </c>
-      <c r="B4">
-        <v>121212</v>
-      </c>
-      <c r="C4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D4" s="4">
-        <v>46281.000972222224</v>
-      </c>
-      <c r="E4" t="s">
-        <v>89</v>
-      </c>
-      <c r="F4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D7" s="4"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D8" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1434,7 +1426,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16" customWidth="1"/>
@@ -1601,6 +1593,56 @@
         <v>49</v>
       </c>
     </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1231234</v>
+      </c>
+      <c r="B4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" s="3">
+        <v>46276</v>
+      </c>
+      <c r="F4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4" s="4">
+        <v>46276.529479166667</v>
+      </c>
+      <c r="J4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K4" s="4">
+        <v>46282.215011574073</v>
+      </c>
+      <c r="L4" t="s">
+        <v>49</v>
+      </c>
+      <c r="M4" t="s">
+        <v>96</v>
+      </c>
+      <c r="N4" s="4">
+        <v>46282.215011574073</v>
+      </c>
+      <c r="O4" s="4">
+        <v>46282.215567129628</v>
+      </c>
+      <c r="P4" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1609,7 +1651,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="16" customWidth="1"/>
@@ -1848,6 +1890,110 @@
         <v>46282.194918981484</v>
       </c>
       <c r="H9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>1231234</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="4">
+        <v>46282.21471064815</v>
+      </c>
+      <c r="E10" t="s">
+        <v>94</v>
+      </c>
+      <c r="F10" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="4">
+        <v>46282.215567129628</v>
+      </c>
+      <c r="H10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <v>1231234</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="4">
+        <v>46282.214791666665</v>
+      </c>
+      <c r="E11" t="s">
+        <v>95</v>
+      </c>
+      <c r="F11" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" s="4">
+        <v>46282.215567129628</v>
+      </c>
+      <c r="H11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>1231234</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="4">
+        <v>46282.214861111112</v>
+      </c>
+      <c r="E12" t="s">
+        <v>94</v>
+      </c>
+      <c r="F12" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" s="4">
+        <v>46282.215567129628</v>
+      </c>
+      <c r="H12" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <v>1231234</v>
+      </c>
+      <c r="C13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="4">
+        <v>46282.215011574073</v>
+      </c>
+      <c r="E13" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" t="s">
+        <v>53</v>
+      </c>
+      <c r="G13" s="4">
+        <v>46282.215567129628</v>
+      </c>
+      <c r="H13" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>